<commit_message>
QCMS v4.13.7 - supply purchase orders, FSI part identity and approved RMTC worksheets
</commit_message>
<xml_diff>
--- a/templates/Part_Master_Template.xlsx
+++ b/templates/Part_Master_Template.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Part Header" sheetId="1" r:id="R943551a081b24041"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Material Details" sheetId="2" r:id="Rafa2ad8d62f04df0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jominy Requirement" sheetId="3" r:id="R44d82ee6288345fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heat Treatment Details" sheetId="4" r:id="Rfb6c8a0a93c646b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Part Header" sheetId="1" r:id="R7fccbadcd7b84c8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Material Details" sheetId="2" r:id="R1e033be24a184a78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jominy Requirement" sheetId="3" r:id="R0be0780aa3fc4ed9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heat Treatment Details" sheetId="4" r:id="R44f5175579fb47b4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -219,9 +219,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -352,62 +352,48 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="18" customWidth="1"/>
-    <x:col min="2" max="2" width="28" customWidth="1"/>
-    <x:col min="3" max="3" width="24" customWidth="1"/>
-    <x:col min="4" max="4" width="18" customWidth="1"/>
-    <x:col min="5" max="5" width="20" customWidth="1"/>
-    <x:col min="6" max="6" width="20" customWidth="1"/>
-    <x:col min="7" max="7" width="16" customWidth="1"/>
-    <x:col min="8" max="8" width="14" customWidth="1"/>
-    <x:col min="9" max="9" width="30" customWidth="1"/>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="23" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="30" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Part Number</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Part Description</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Customer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Material Grade</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Part Finish Weight kg</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Drawing Number</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Drawing Revision</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Status</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Remarks</x:t>
-        </x:is>
+      <x:c r="A1" s="1" t="str">
+        <x:v>Part Number</x:v>
+      </x:c>
+      <x:c r="B1" s="1" t="str">
+        <x:v>FSI Part Number</x:v>
+      </x:c>
+      <x:c r="C1" s="1" t="str">
+        <x:v>Part Description</x:v>
+      </x:c>
+      <x:c r="D1" s="1" t="str">
+        <x:v>Customer</x:v>
+      </x:c>
+      <x:c r="E1" s="1" t="str">
+        <x:v>Material Grade</x:v>
+      </x:c>
+      <x:c r="F1" s="1" t="str">
+        <x:v>Part Finish Weight kg</x:v>
+      </x:c>
+      <x:c r="G1" s="1" t="str">
+        <x:v>Drawing Number</x:v>
+      </x:c>
+      <x:c r="H1" s="1" t="str">
+        <x:v>Drawing Revision</x:v>
+      </x:c>
+      <x:c r="I1" s="1" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="J1" t="str">
+        <x:v>Remarks</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -416,46 +402,19 @@
           <x:t xml:space="preserve"/>
         </x:is>
       </x:c>
-      <x:c r="B2" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="C2" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="D2" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="E2" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="F2" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="G2" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="H2" s="2" t="inlineStr">
+      <x:c r="B2" s="2" t="str"/>
+      <x:c r="C2" s="2"/>
+      <x:c r="D2" s="2"/>
+      <x:c r="E2" s="2"/>
+      <x:c r="F2" s="2"/>
+      <x:c r="G2" s="2"/>
+      <x:c r="H2" s="2"/>
+      <x:c r="I2" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">ACTIVE</x:t>
         </x:is>
       </x:c>
-      <x:c r="I2" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="J2"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>